<commit_message>
feat: dataset completo de 16 activos industriales, tarjetas tecnicas y QRs
</commit_message>
<xml_diff>
--- a/inventario_activos.xlsx
+++ b/inventario_activos.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X7"/>
+  <dimension ref="A1:X17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -646,19 +646,19 @@
       </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t>2026-09-17 10:01:15</t>
+          <t>2026-09-17 10:27:53</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>DBL-PRE-001</t>
+          <t>MAQ-PRN-001</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Plegadora Dobladora CNC Hidráulica 175T</t>
+          <t>Punzonadora CNC de Alta Frecuencia 300kN</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -668,12 +668,12 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>TruBend 5170</t>
+          <t>TruPunch 5000 S12</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>TB-5170-8834</t>
+          <t>TP-5000-4491</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -683,12 +683,12 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Dobladora</t>
+          <t>Punzonadora CNC</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>B7C91142-990A-4E32-B871-33C29910D442</t>
+          <t>5B2E9D34-78CD-55A2-A3FB-2B9C4678E112</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -706,39 +706,39 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>23 16 3840 7002044</t>
+          <t>23 16 3840 7002554</t>
         </is>
       </c>
       <c r="M3" t="n">
-        <v>3420000</v>
+        <v>4150000</v>
       </c>
       <c r="N3" t="n">
-        <v>145000</v>
+        <v>180000</v>
       </c>
       <c r="O3" t="n">
-        <v>3565000</v>
+        <v>4330000</v>
       </c>
       <c r="P3" t="n">
         <v>10</v>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>2023-06-20</t>
+          <t>2023-05-10</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>2023-07-05</t>
+          <t>2023-05-25</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>Doblez</t>
+          <t>Corte</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>Téc. Roberto Garza</t>
+          <t>Ing. Carlos Mendoza</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
@@ -748,64 +748,64 @@
       </c>
       <c r="V3" t="inlineStr">
         <is>
-          <t>media/fotos_activos/DBL-PRE-001.jpg</t>
+          <t>media/fotos_activos/MAQ-PRN-001.jpg</t>
         </is>
       </c>
       <c r="W3" t="inlineStr">
         <is>
-          <t>media/qrs/QR_DBL-PRE-001.png</t>
+          <t>media/qrs/QR_MAQ-PRN-001.png</t>
         </is>
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>2026-09-17 10:01:15</t>
+          <t>2026-09-17 10:27:53</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>PNT-BAT-001</t>
+          <t>LIJ-REB-001</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Cabina de Pintura Electrostática en Polvo</t>
+          <t>Lijadora y Rebabeadora Automática de Bordes</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Wagner</t>
+          <t>Timesavers</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>SuperCube Quick-Clean</t>
+          <t>42 Series Rotary Brush</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>WG-SC-2022-09</t>
+          <t>TS-42-8821-B</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Línea de Pintura</t>
+          <t>Maquinaria Principal</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Pintura Batch</t>
+          <t>Lijadora/Rebabeadora</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>9F10DE32-3401-44B8-B590-AA382109CC11</t>
+          <t>8C3F0E45-89DE-66B3-B4AC-3C0D5789F223</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>WAG881120AB9</t>
+          <t>TSA100214KJ3</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
@@ -814,39 +814,43 @@
         </is>
       </c>
       <c r="K4" t="b">
-        <v>0</v>
-      </c>
-      <c r="L4" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>23 16 3840 7003118</t>
+        </is>
+      </c>
       <c r="M4" t="n">
-        <v>1890000</v>
+        <v>1280000</v>
       </c>
       <c r="N4" t="n">
-        <v>98000</v>
+        <v>65000</v>
       </c>
       <c r="O4" t="n">
-        <v>1988000</v>
+        <v>1345000</v>
       </c>
       <c r="P4" t="n">
         <v>10</v>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>2022-11-10</t>
+          <t>2023-08-14</t>
         </is>
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>2022-12-01</t>
+          <t>2023-09-01</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>Pintura</t>
+          <t>Corte</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>Ing. Sofía Valdés</t>
+          <t>Téc. Javier Ortiz</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
@@ -856,64 +860,64 @@
       </c>
       <c r="V4" t="inlineStr">
         <is>
-          <t>media/fotos_activos/PNT-BAT-001.jpg</t>
+          <t>media/fotos_activos/LIJ-REB-001.jpg</t>
         </is>
       </c>
       <c r="W4" t="inlineStr">
         <is>
-          <t>media/qrs/QR_PNT-BAT-001.png</t>
+          <t>media/qrs/QR_LIJ-REB-001.png</t>
         </is>
       </c>
       <c r="X4" t="inlineStr">
         <is>
-          <t>2026-09-17 10:01:15</t>
+          <t>2026-09-17 10:27:54</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>EQM-MTC-001</t>
+          <t>DBL-PRE-001</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Montacargas Eléctrico Hombre Sentado 2.5T</t>
+          <t>Plegadora Dobladora CNC Hidráulica 175T</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Toyota / Raymond</t>
+          <t>Trumpf</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>8FBE20</t>
+          <t>TruBend 5170</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>TY-8FBE-99120</t>
+          <t>TB-5170-8834</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Equipo Móvil</t>
+          <t>Maquinaria Principal</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Montacargas</t>
+          <t>Dobladora</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>88A3CD19-4500-4762-AC81-6543209EE890</t>
+          <t>B7C91142-990A-4E32-B871-33C29910D442</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>TMX950812GH4</t>
+          <t>TRU020511RT8</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
@@ -922,39 +926,43 @@
         </is>
       </c>
       <c r="K5" t="b">
-        <v>0</v>
-      </c>
-      <c r="L5" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>23 16 3840 7002044</t>
+        </is>
+      </c>
       <c r="M5" t="n">
-        <v>850000</v>
+        <v>3420000</v>
       </c>
       <c r="N5" t="n">
-        <v>25000</v>
+        <v>145000</v>
       </c>
       <c r="O5" t="n">
-        <v>875000</v>
+        <v>3565000</v>
       </c>
       <c r="P5" t="n">
-        <v>25</v>
+        <v>10</v>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>2024-01-15</t>
+          <t>2023-06-20</t>
         </is>
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>2024-01-20</t>
+          <t>2023-07-05</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>Logística</t>
+          <t>Doblez</t>
         </is>
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>Miguel Ángel Rivas</t>
+          <t>Téc. Roberto Garza</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
@@ -964,69 +972,69 @@
       </c>
       <c r="V5" t="inlineStr">
         <is>
-          <t>media/fotos_activos/EQM-MTC-001.jpg</t>
+          <t>media/fotos_activos/DBL-PRE-001.jpg</t>
         </is>
       </c>
       <c r="W5" t="inlineStr">
         <is>
-          <t>media/qrs/QR_EQM-MTC-001.png</t>
+          <t>media/qrs/QR_DBL-PRE-001.png</t>
         </is>
       </c>
       <c r="X5" t="inlineStr">
         <is>
-          <t>2026-09-17 10:01:15</t>
+          <t>2026-09-17 10:27:54</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>HRR-PUN-001</t>
+          <t>DBL-PRE-002</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Juego de Punzón y Dados de Alta Precisión R1</t>
+          <t>Dobladora Eléctrica Servodrive 40T</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Wila</t>
+          <t>Amada</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>New Standard Pro Tooling</t>
+          <t>EG 4010 Compact</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>WL-PUN-0918-X</t>
+          <t>AM-EG-4010-09</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Herramental de Doblez</t>
+          <t>Maquinaria Principal</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Dado/Punzón</t>
+          <t>Dobladora</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>3C871A02-B891-45FE-8711-2290CDA10988</t>
+          <t>6D4A1F56-90EF-77C4-C5BD-4D1E6890A334</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>WIL120405NM1</t>
+          <t>AMD910620LK9</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>I05 Dados, troqueles, moldes, matrices y herramental</t>
+          <t>I02 Maquinaria y equipo</t>
         </is>
       </c>
       <c r="K6" t="b">
@@ -1034,29 +1042,29 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>24 16 3840 8000412</t>
+          <t>24 16 3840 8001102</t>
         </is>
       </c>
       <c r="M6" t="n">
-        <v>260000</v>
+        <v>1950000</v>
       </c>
       <c r="N6" t="n">
-        <v>15000</v>
+        <v>82000</v>
       </c>
       <c r="O6" t="n">
-        <v>275000</v>
+        <v>2032000</v>
       </c>
       <c r="P6" t="n">
-        <v>35</v>
+        <v>10</v>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>2024-02-10</t>
+          <t>2024-01-18</t>
         </is>
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>2024-02-15</t>
+          <t>2024-02-01</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
@@ -1071,130 +1079,1234 @@
       </c>
       <c r="U6" t="inlineStr">
         <is>
-          <t>Crítico</t>
+          <t>Operativo</t>
         </is>
       </c>
       <c r="V6" t="inlineStr">
         <is>
-          <t>media/fotos_activos/HRR-PUN-001.jpg</t>
+          <t>media/fotos_activos/DBL-PRE-002.jpg</t>
         </is>
       </c>
       <c r="W6" t="inlineStr">
         <is>
-          <t>media/qrs/QR_HRR-PUN-001.png</t>
+          <t>media/qrs/QR_DBL-PRE-002.png</t>
         </is>
       </c>
       <c r="X6" t="inlineStr">
         <is>
-          <t>2026-09-17 10:01:16</t>
+          <t>2026-09-17 10:27:54</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
+          <t>HRR-PUN-001</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Juego de Punzón y Dados de Alta Precisión R1</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Wila</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>New Standard Pro Tooling</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>WL-PUN-0918-X</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Herramental de Doblez</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Dado/Punzón</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>3C871A02-B891-45FE-8711-2290CDA10988</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>WIL120405NM1</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>I05 Dados, troqueles, moldes, matrices y herramental</t>
+        </is>
+      </c>
+      <c r="K7" t="b">
+        <v>1</v>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>24 16 3840 8000412</t>
+        </is>
+      </c>
+      <c r="M7" t="n">
+        <v>260000</v>
+      </c>
+      <c r="N7" t="n">
+        <v>15000</v>
+      </c>
+      <c r="O7" t="n">
+        <v>275000</v>
+      </c>
+      <c r="P7" t="n">
+        <v>35</v>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>2024-02-10</t>
+        </is>
+      </c>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>2024-02-15</t>
+        </is>
+      </c>
+      <c r="S7" t="inlineStr">
+        <is>
+          <t>Doblez</t>
+        </is>
+      </c>
+      <c r="T7" t="inlineStr">
+        <is>
+          <t>Téc. Roberto Garza</t>
+        </is>
+      </c>
+      <c r="U7" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+      <c r="V7" t="inlineStr">
+        <is>
+          <t>media/fotos_activos/HRR-PUN-001.jpg</t>
+        </is>
+      </c>
+      <c r="W7" t="inlineStr">
+        <is>
+          <t>media/qrs/QR_HRR-PUN-001.png</t>
+        </is>
+      </c>
+      <c r="X7" t="inlineStr">
+        <is>
+          <t>2026-09-17 10:27:54</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>HRR-DBL-001</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Matriz Multivía de Cambio Rápido V8-V24</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Rolleri</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>R1 Multi-V Die Type</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>ROL-MV-2024</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Herramental de Doblez</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Matriz Multivía</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>7E5B2A67-01FA-88D5-D6CE-5E2F7901B445</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>ROL080312GH8</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>I05 Dados, troqueles, moldes, matrices y herramental</t>
+        </is>
+      </c>
+      <c r="K8" t="b">
+        <v>1</v>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>24 16 3840 8001990</t>
+        </is>
+      </c>
+      <c r="M8" t="n">
+        <v>185000</v>
+      </c>
+      <c r="N8" t="n">
+        <v>12000</v>
+      </c>
+      <c r="O8" t="n">
+        <v>197000</v>
+      </c>
+      <c r="P8" t="n">
+        <v>35</v>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>2024-03-05</t>
+        </is>
+      </c>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>2024-03-10</t>
+        </is>
+      </c>
+      <c r="S8" t="inlineStr">
+        <is>
+          <t>Doblez</t>
+        </is>
+      </c>
+      <c r="T8" t="inlineStr">
+        <is>
+          <t>Téc. Roberto Garza</t>
+        </is>
+      </c>
+      <c r="U8" t="inlineStr">
+        <is>
+          <t>Operativo</t>
+        </is>
+      </c>
+      <c r="V8" t="inlineStr">
+        <is>
+          <t>media/fotos_activos/HRR-DBL-001.jpg</t>
+        </is>
+      </c>
+      <c r="W8" t="inlineStr">
+        <is>
+          <t>media/qrs/QR_HRR-DBL-001.png</t>
+        </is>
+      </c>
+      <c r="X8" t="inlineStr">
+        <is>
+          <t>2026-09-17 10:27:54</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>PNT-BAT-001</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Cabina de Pintura Electrostática en Polvo</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Wagner</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>SuperCube Quick-Clean</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>WG-SC-2022-09</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Línea de Pintura</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Pintura Batch</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>9F10DE32-3401-44B8-B590-AA382109CC11</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>WAG881120AB9</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>I02 Maquinaria y equipo</t>
+        </is>
+      </c>
+      <c r="K9" t="b">
+        <v>0</v>
+      </c>
+      <c r="L9" t="inlineStr"/>
+      <c r="M9" t="n">
+        <v>1890000</v>
+      </c>
+      <c r="N9" t="n">
+        <v>98000</v>
+      </c>
+      <c r="O9" t="n">
+        <v>1988000</v>
+      </c>
+      <c r="P9" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>2022-11-10</t>
+        </is>
+      </c>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>2022-12-01</t>
+        </is>
+      </c>
+      <c r="S9" t="inlineStr">
+        <is>
+          <t>Pintura</t>
+        </is>
+      </c>
+      <c r="T9" t="inlineStr">
+        <is>
+          <t>Ing. Sofía Valdés</t>
+        </is>
+      </c>
+      <c r="U9" t="inlineStr">
+        <is>
+          <t>Operativo</t>
+        </is>
+      </c>
+      <c r="V9" t="inlineStr">
+        <is>
+          <t>media/fotos_activos/PNT-BAT-001.jpg</t>
+        </is>
+      </c>
+      <c r="W9" t="inlineStr">
+        <is>
+          <t>media/qrs/QR_PNT-BAT-001.png</t>
+        </is>
+      </c>
+      <c r="X9" t="inlineStr">
+        <is>
+          <t>2026-09-17 10:27:55</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>PNT-LIN-001</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Horno Convectivo de Curado de Pintura 220°C</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Blowtherm Industrial</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>ThermoCure 6000 Gas</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>BLW-TC-220-41</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Línea de Pintura</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Horno de Curado</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>8F6C3B78-12AB-99E6-E7DF-6F3A8012C556</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>BLW050720RT2</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>I02 Maquinaria y equipo</t>
+        </is>
+      </c>
+      <c r="K10" t="b">
+        <v>1</v>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>23 16 3840 7004012</t>
+        </is>
+      </c>
+      <c r="M10" t="n">
+        <v>2450000</v>
+      </c>
+      <c r="N10" t="n">
+        <v>110000</v>
+      </c>
+      <c r="O10" t="n">
+        <v>2560000</v>
+      </c>
+      <c r="P10" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>2023-02-22</t>
+        </is>
+      </c>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>2023-03-10</t>
+        </is>
+      </c>
+      <c r="S10" t="inlineStr">
+        <is>
+          <t>Pintura</t>
+        </is>
+      </c>
+      <c r="T10" t="inlineStr">
+        <is>
+          <t>Ing. Sofía Valdés</t>
+        </is>
+      </c>
+      <c r="U10" t="inlineStr">
+        <is>
+          <t>Operativo</t>
+        </is>
+      </c>
+      <c r="V10" t="inlineStr">
+        <is>
+          <t>media/fotos_activos/PNT-LIN-001.jpg</t>
+        </is>
+      </c>
+      <c r="W10" t="inlineStr">
+        <is>
+          <t>media/qrs/QR_PNT-LIN-001.png</t>
+        </is>
+      </c>
+      <c r="X10" t="inlineStr">
+        <is>
+          <t>2026-09-17 10:27:55</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>HRR-MAN-001</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Pistolas Electrostáticas de Aplicación Manual</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Nordson</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Encore HD Spray System</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>ND-ENC-2024-03</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Herramienta de Mano</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Pistola de Torque</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>9A7D4C89-23BC-00F7-F8EA-7A4B9123D667</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>NDS990412MK1</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>I02 Maquinaria y equipo</t>
+        </is>
+      </c>
+      <c r="K11" t="b">
+        <v>1</v>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>24 16 3840 8002230</t>
+        </is>
+      </c>
+      <c r="M11" t="n">
+        <v>165000</v>
+      </c>
+      <c r="N11" t="n">
+        <v>8500</v>
+      </c>
+      <c r="O11" t="n">
+        <v>173500</v>
+      </c>
+      <c r="P11" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>2024-03-12</t>
+        </is>
+      </c>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>2024-03-15</t>
+        </is>
+      </c>
+      <c r="S11" t="inlineStr">
+        <is>
+          <t>Pintura</t>
+        </is>
+      </c>
+      <c r="T11" t="inlineStr">
+        <is>
+          <t>Téc. Andrés Lozano</t>
+        </is>
+      </c>
+      <c r="U11" t="inlineStr">
+        <is>
+          <t>En Mantenimiento</t>
+        </is>
+      </c>
+      <c r="V11" t="inlineStr">
+        <is>
+          <t>media/fotos_activos/HRR-MAN-001.jpg</t>
+        </is>
+      </c>
+      <c r="W11" t="inlineStr">
+        <is>
+          <t>media/qrs/QR_HRR-MAN-001.png</t>
+        </is>
+      </c>
+      <c r="X11" t="inlineStr">
+        <is>
+          <t>2026-09-17 10:27:55</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
           <t>EST-MES-001</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Estación Ergonomica de Ensamble y Remachado</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Estación Ergonómica de Ensamble y Remachado</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
         <is>
           <t>Bosch Rexroth</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="D12" t="inlineStr">
         <is>
           <t>EcoSafe Modular Workstation</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="E12" t="inlineStr">
         <is>
           <t>BR-WS-1142</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
+      <c r="F12" t="inlineStr">
         <is>
           <t>Estaciones/Mesas</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr">
+      <c r="G12" t="inlineStr">
         <is>
           <t>Mesa</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr">
+      <c r="H12" t="inlineStr">
         <is>
           <t>77D89C11-0022-498A-9877-1122AA990022</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr">
+      <c r="I12" t="inlineStr">
         <is>
           <t>BRE010915TR3</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr">
+      <c r="J12" t="inlineStr">
         <is>
           <t>I02 Maquinaria y equipo</t>
         </is>
       </c>
-      <c r="K7" t="b">
+      <c r="K12" t="b">
         <v>0</v>
       </c>
-      <c r="L7" t="inlineStr"/>
-      <c r="M7" t="n">
+      <c r="L12" t="inlineStr"/>
+      <c r="M12" t="n">
         <v>145000</v>
       </c>
-      <c r="N7" t="n">
+      <c r="N12" t="n">
         <v>8000</v>
       </c>
-      <c r="O7" t="n">
+      <c r="O12" t="n">
         <v>153000</v>
       </c>
-      <c r="P7" t="n">
+      <c r="P12" t="n">
         <v>10</v>
       </c>
-      <c r="Q7" t="inlineStr">
+      <c r="Q12" t="inlineStr">
         <is>
           <t>2024-04-05</t>
         </is>
       </c>
-      <c r="R7" t="inlineStr">
+      <c r="R12" t="inlineStr">
         <is>
           <t>2024-04-10</t>
         </is>
       </c>
-      <c r="S7" t="inlineStr">
+      <c r="S12" t="inlineStr">
         <is>
           <t>Ensamblado</t>
         </is>
       </c>
-      <c r="T7" t="inlineStr">
+      <c r="T12" t="inlineStr">
         <is>
           <t>Téc. Laura Domínguez</t>
         </is>
       </c>
-      <c r="U7" t="inlineStr">
+      <c r="U12" t="inlineStr">
         <is>
           <t>Operativo</t>
         </is>
       </c>
-      <c r="V7" t="inlineStr">
+      <c r="V12" t="inlineStr">
         <is>
           <t>media/fotos_activos/EST-MES-001.jpg</t>
         </is>
       </c>
-      <c r="W7" t="inlineStr">
+      <c r="W12" t="inlineStr">
         <is>
           <t>media/qrs/QR_EST-MES-001.png</t>
         </is>
       </c>
-      <c r="X7" t="inlineStr">
-        <is>
-          <t>2026-09-17 10:01:16</t>
+      <c r="X12" t="inlineStr">
+        <is>
+          <t>2026-09-17 10:27:55</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>EST-EST-001</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Mesa 3D de Sujeción y Soldadura 2000x1000mm</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Siegmund</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>System 28 Professional 750</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>SG-28-200100</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Estaciones/Mesas</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Estación de Soldadura</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>0B8E5D90-34CD-11A8-A9FB-8B5C0234E778</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>SGM110825GH3</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>I02 Maquinaria y equipo</t>
+        </is>
+      </c>
+      <c r="K13" t="b">
+        <v>1</v>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>24 16 3840 8003112</t>
+        </is>
+      </c>
+      <c r="M13" t="n">
+        <v>210000</v>
+      </c>
+      <c r="N13" t="n">
+        <v>14000</v>
+      </c>
+      <c r="O13" t="n">
+        <v>224000</v>
+      </c>
+      <c r="P13" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q13" t="inlineStr">
+        <is>
+          <t>2024-04-12</t>
+        </is>
+      </c>
+      <c r="R13" t="inlineStr">
+        <is>
+          <t>2024-04-18</t>
+        </is>
+      </c>
+      <c r="S13" t="inlineStr">
+        <is>
+          <t>Ensamblado</t>
+        </is>
+      </c>
+      <c r="T13" t="inlineStr">
+        <is>
+          <t>Téc. Laura Domínguez</t>
+        </is>
+      </c>
+      <c r="U13" t="inlineStr">
+        <is>
+          <t>Operativo</t>
+        </is>
+      </c>
+      <c r="V13" t="inlineStr">
+        <is>
+          <t>media/fotos_activos/EST-EST-001.jpg</t>
+        </is>
+      </c>
+      <c r="W13" t="inlineStr">
+        <is>
+          <t>media/qrs/QR_EST-EST-001.png</t>
+        </is>
+      </c>
+      <c r="X13" t="inlineStr">
+        <is>
+          <t>2026-09-17 10:27:55</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>MAQ-PRN-002</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Celda Robotizada de Soldadura Mig/Mag</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>KUKA / Fronius</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>KR CYBERTECH nano + TPS 400i</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>KK-CYB-2023-11</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Maquinaria Principal</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Otra Maquinaria Principal</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>1C9F6E01-45DE-22B9-B0AC-9C6D1345F889</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>KUK040319TY5</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>I02 Maquinaria y equipo</t>
+        </is>
+      </c>
+      <c r="K14" t="b">
+        <v>1</v>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>23 16 3840 7005882</t>
+        </is>
+      </c>
+      <c r="M14" t="n">
+        <v>3650000</v>
+      </c>
+      <c r="N14" t="n">
+        <v>195000</v>
+      </c>
+      <c r="O14" t="n">
+        <v>3845000</v>
+      </c>
+      <c r="P14" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q14" t="inlineStr">
+        <is>
+          <t>2023-10-02</t>
+        </is>
+      </c>
+      <c r="R14" t="inlineStr">
+        <is>
+          <t>2023-11-15</t>
+        </is>
+      </c>
+      <c r="S14" t="inlineStr">
+        <is>
+          <t>Ensamblado</t>
+        </is>
+      </c>
+      <c r="T14" t="inlineStr">
+        <is>
+          <t>Ing. Carlos Mendoza</t>
+        </is>
+      </c>
+      <c r="U14" t="inlineStr">
+        <is>
+          <t>Operativo</t>
+        </is>
+      </c>
+      <c r="V14" t="inlineStr">
+        <is>
+          <t>media/fotos_activos/MAQ-PRN-002.jpg</t>
+        </is>
+      </c>
+      <c r="W14" t="inlineStr">
+        <is>
+          <t>media/qrs/QR_MAQ-PRN-002.png</t>
+        </is>
+      </c>
+      <c r="X14" t="inlineStr">
+        <is>
+          <t>2026-09-17 10:27:56</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>HRR-MAN-002</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Remachadora Neumática Industrial de Alta Fuerza</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Lobster</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>R1A1 Heavy Duty</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>LOB-R1A1-901</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Herramienta de Mano</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Remachadora Neumática</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>2D0A7F12-56EF-33CA-C1BD-0D7E2456A990</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>LOB140210VB7</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>I02 Maquinaria y equipo</t>
+        </is>
+      </c>
+      <c r="K15" t="b">
+        <v>0</v>
+      </c>
+      <c r="L15" t="inlineStr"/>
+      <c r="M15" t="n">
+        <v>48000</v>
+      </c>
+      <c r="N15" t="n">
+        <v>2500</v>
+      </c>
+      <c r="O15" t="n">
+        <v>50500</v>
+      </c>
+      <c r="P15" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q15" t="inlineStr">
+        <is>
+          <t>2024-05-10</t>
+        </is>
+      </c>
+      <c r="R15" t="inlineStr">
+        <is>
+          <t>2024-05-12</t>
+        </is>
+      </c>
+      <c r="S15" t="inlineStr">
+        <is>
+          <t>Ensamblado</t>
+        </is>
+      </c>
+      <c r="T15" t="inlineStr">
+        <is>
+          <t>Téc. Laura Domínguez</t>
+        </is>
+      </c>
+      <c r="U15" t="inlineStr">
+        <is>
+          <t>Operativo</t>
+        </is>
+      </c>
+      <c r="V15" t="inlineStr">
+        <is>
+          <t>media/fotos_activos/HRR-MAN-002.jpg</t>
+        </is>
+      </c>
+      <c r="W15" t="inlineStr">
+        <is>
+          <t>media/qrs/QR_HRR-MAN-002.png</t>
+        </is>
+      </c>
+      <c r="X15" t="inlineStr">
+        <is>
+          <t>2026-09-17 10:27:56</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>EQM-MTC-001</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Montacargas Eléctrico Hombre Sentado 2.5T</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Toyota / Raymond</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>8FBE20</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>TY-8FBE-99120</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Equipo Móvil</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Montacargas</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>88A3CD19-4500-4762-AC81-6543209EE890</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>TMX950812GH4</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>I02 Maquinaria y equipo</t>
+        </is>
+      </c>
+      <c r="K16" t="b">
+        <v>0</v>
+      </c>
+      <c r="L16" t="inlineStr"/>
+      <c r="M16" t="n">
+        <v>850000</v>
+      </c>
+      <c r="N16" t="n">
+        <v>25000</v>
+      </c>
+      <c r="O16" t="n">
+        <v>875000</v>
+      </c>
+      <c r="P16" t="n">
+        <v>25</v>
+      </c>
+      <c r="Q16" t="inlineStr">
+        <is>
+          <t>2024-01-15</t>
+        </is>
+      </c>
+      <c r="R16" t="inlineStr">
+        <is>
+          <t>2024-01-20</t>
+        </is>
+      </c>
+      <c r="S16" t="inlineStr">
+        <is>
+          <t>Logística</t>
+        </is>
+      </c>
+      <c r="T16" t="inlineStr">
+        <is>
+          <t>Miguel Ángel Rivas</t>
+        </is>
+      </c>
+      <c r="U16" t="inlineStr">
+        <is>
+          <t>Operativo</t>
+        </is>
+      </c>
+      <c r="V16" t="inlineStr">
+        <is>
+          <t>media/fotos_activos/EQM-MTC-001.jpg</t>
+        </is>
+      </c>
+      <c r="W16" t="inlineStr">
+        <is>
+          <t>media/qrs/QR_EQM-MTC-001.png</t>
+        </is>
+      </c>
+      <c r="X16" t="inlineStr">
+        <is>
+          <t>2026-09-17 10:27:56</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>EQM-PTH-001</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Patín Hidráulico de Carga Pesada 3T</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Crown</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>PTH 50 Series 6000lbs</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>CRW-PTH-3301</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Equipo Móvil</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Patín Hidráulico</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>3E1B8A23-67FA-44DB-D2CE-1E8F3567B001</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>CRW030615NM4</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>I02 Maquinaria y equipo</t>
+        </is>
+      </c>
+      <c r="K17" t="b">
+        <v>0</v>
+      </c>
+      <c r="L17" t="inlineStr"/>
+      <c r="M17" t="n">
+        <v>32000</v>
+      </c>
+      <c r="N17" t="n">
+        <v>1800</v>
+      </c>
+      <c r="O17" t="n">
+        <v>33800</v>
+      </c>
+      <c r="P17" t="n">
+        <v>25</v>
+      </c>
+      <c r="Q17" t="inlineStr">
+        <is>
+          <t>2024-02-28</t>
+        </is>
+      </c>
+      <c r="R17" t="inlineStr">
+        <is>
+          <t>2024-03-01</t>
+        </is>
+      </c>
+      <c r="S17" t="inlineStr">
+        <is>
+          <t>Logística</t>
+        </is>
+      </c>
+      <c r="T17" t="inlineStr">
+        <is>
+          <t>Miguel Ángel Rivas</t>
+        </is>
+      </c>
+      <c r="U17" t="inlineStr">
+        <is>
+          <t>Operativo</t>
+        </is>
+      </c>
+      <c r="V17" t="inlineStr">
+        <is>
+          <t>media/fotos_activos/EQM-PTH-001.jpg</t>
+        </is>
+      </c>
+      <c r="W17" t="inlineStr">
+        <is>
+          <t>media/qrs/QR_EQM-PTH-001.png</t>
+        </is>
+      </c>
+      <c r="X17" t="inlineStr">
+        <is>
+          <t>2026-09-17 10:27:56</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: migracion e importacion de 14 activos reales y fotografias de planta desde ACTIVOS.accdb
</commit_message>
<xml_diff>
--- a/inventario_activos.xlsx
+++ b/inventario_activos.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X1"/>
+  <dimension ref="A1:X15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -535,6 +535,1546 @@
       <c r="X1" t="inlineStr">
         <is>
           <t>Fecha_Registro</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>CTR-LAS-001</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Máquina de Corte Láser CNC 1 (NOVA3015)</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>FLEXMAX</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>NOVA3015</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>52J-0135</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Maquinaria Principal</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Corte Láser</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>4A1E8D23-67BC-44F1-92EA-CTRLAS001</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>FCM180614LK2</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>I02 Maquinaria y equipo</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="n">
+        <v>536385.75</v>
+      </c>
+      <c r="N2" t="n">
+        <v>26819.29</v>
+      </c>
+      <c r="O2" t="n">
+        <v>563205.04</v>
+      </c>
+      <c r="P2" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>2025-12-16</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>2025-12-16</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>Corte</t>
+        </is>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>Ing. Carlos Mendoza</t>
+        </is>
+      </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>Operativo</t>
+        </is>
+      </c>
+      <c r="V2" t="inlineStr">
+        <is>
+          <t>media/fotos_activos/CTR-LAS-001.jpg</t>
+        </is>
+      </c>
+      <c r="W2" t="inlineStr">
+        <is>
+          <t>media/qrs/QR_CTR-LAS-001.png</t>
+        </is>
+      </c>
+      <c r="X2" t="inlineStr">
+        <is>
+          <t>2026-09-17 13:02</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>CTR-LAS-002</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Máquina de Corte Láser CNC 2 (NOVA3015)</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>FLEXMAX</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>NOVA3015</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>52J-0133</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Maquinaria Principal</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Corte Láser</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>4A1E8D23-67BC-44F1-92EA-CTRLAS002</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>FCM180614LK2</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>I02 Maquinaria y equipo</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="n">
+        <v>536385.75</v>
+      </c>
+      <c r="N3" t="n">
+        <v>26819.29</v>
+      </c>
+      <c r="O3" t="n">
+        <v>563205.04</v>
+      </c>
+      <c r="P3" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>2025-12-16</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>2025-12-16</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>Corte</t>
+        </is>
+      </c>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>Ing. Carlos Mendoza</t>
+        </is>
+      </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>Operativo</t>
+        </is>
+      </c>
+      <c r="V3" t="inlineStr">
+        <is>
+          <t>media/fotos_activos/CTR-LAS-002.jpg</t>
+        </is>
+      </c>
+      <c r="W3" t="inlineStr">
+        <is>
+          <t>media/qrs/QR_CTR-LAS-002.png</t>
+        </is>
+      </c>
+      <c r="X3" t="inlineStr">
+        <is>
+          <t>2026-09-17 13:02</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>EQM-CMP-002</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Compresor de Tornillo Industrial 2</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>BOSSDREI</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>BCT-3022-SET/BCS-TR03</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>SD0012502-04502</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Herramientas y Periféricos</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Compresor Industrial</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>4A1E8D23-67BC-44F1-92EA-EQMCMP002</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>FCM180614LK2</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>I02 Maquinaria y equipo</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="n">
+        <v>235425</v>
+      </c>
+      <c r="N4" t="n">
+        <v>11771.25</v>
+      </c>
+      <c r="O4" t="n">
+        <v>247196.25</v>
+      </c>
+      <c r="P4" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>2025-12-16</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>2025-12-16</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>Corte</t>
+        </is>
+      </c>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>Téc. Roberto Garza</t>
+        </is>
+      </c>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>Operativo</t>
+        </is>
+      </c>
+      <c r="V4" t="inlineStr">
+        <is>
+          <t>media/fotos_activos/EQM-CMP-002.jpg</t>
+        </is>
+      </c>
+      <c r="W4" t="inlineStr">
+        <is>
+          <t>media/qrs/QR_EQM-CMP-002.png</t>
+        </is>
+      </c>
+      <c r="X4" t="inlineStr">
+        <is>
+          <t>2026-09-17 13:02</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>EQM-CMP-001</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Compresor de Tornillo Industrial 1</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>BOSSDREI</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>BCT-3022-SET/BCS-TR03</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>SD001-2503-06236</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Herramientas y Periféricos</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Compresor Industrial</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>4A1E8D23-67BC-44F1-92EA-EQMCMP001</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>FCM180614LK2</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>I02 Maquinaria y equipo</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="n">
+        <v>235425</v>
+      </c>
+      <c r="N5" t="n">
+        <v>11771.25</v>
+      </c>
+      <c r="O5" t="n">
+        <v>247196.25</v>
+      </c>
+      <c r="P5" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>2025-12-16</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>2025-12-16</t>
+        </is>
+      </c>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t>Corte</t>
+        </is>
+      </c>
+      <c r="T5" t="inlineStr">
+        <is>
+          <t>Téc. Roberto Garza</t>
+        </is>
+      </c>
+      <c r="U5" t="inlineStr">
+        <is>
+          <t>Operativo</t>
+        </is>
+      </c>
+      <c r="V5" t="inlineStr">
+        <is>
+          <t>media/fotos_activos/EQM-CMP-001.jpg</t>
+        </is>
+      </c>
+      <c r="W5" t="inlineStr">
+        <is>
+          <t>media/qrs/QR_EQM-CMP-001.png</t>
+        </is>
+      </c>
+      <c r="X5" t="inlineStr">
+        <is>
+          <t>2026-09-17 13:02</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>EQM-REG-001</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Regulador de Voltaje Trifásico Láser 1 (60kVA)</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>FLBXON</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>FVR3-60KVA-3P</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>SN-EQM-REG-001</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Herramientas y Periféricos</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Transformador / Regulador</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>4A1E8D23-67BC-44F1-92EA-EQMREG001</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>FCM180614LK2</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>I02 Maquinaria y equipo</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr"/>
+      <c r="M6" t="n">
+        <v>0</v>
+      </c>
+      <c r="N6" t="n">
+        <v>0</v>
+      </c>
+      <c r="O6" t="n">
+        <v>0</v>
+      </c>
+      <c r="P6" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>2025-12-16</t>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>2025-12-16</t>
+        </is>
+      </c>
+      <c r="S6" t="inlineStr">
+        <is>
+          <t>Corte</t>
+        </is>
+      </c>
+      <c r="T6" t="inlineStr">
+        <is>
+          <t>Ing. Fernando Silva</t>
+        </is>
+      </c>
+      <c r="U6" t="inlineStr">
+        <is>
+          <t>Operativo</t>
+        </is>
+      </c>
+      <c r="V6" t="inlineStr">
+        <is>
+          <t>media/fotos_activos/EQM-REG-001.jpg</t>
+        </is>
+      </c>
+      <c r="W6" t="inlineStr">
+        <is>
+          <t>media/qrs/QR_EQM-REG-001.png</t>
+        </is>
+      </c>
+      <c r="X6" t="inlineStr">
+        <is>
+          <t>2026-09-17 13:02</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>EQM-REG-002</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Regulador de Voltaje Trifásico Láser 2 (60kVA)</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>FLBXON</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>FVR3-60KVA-3P</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>SN-EQM-REG-002</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Herramientas y Periféricos</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Transformador / Regulador</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>4A1E8D23-67BC-44F1-92EA-EQMREG002</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>FCM180614LK2</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>I02 Maquinaria y equipo</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr"/>
+      <c r="M7" t="n">
+        <v>0</v>
+      </c>
+      <c r="N7" t="n">
+        <v>0</v>
+      </c>
+      <c r="O7" t="n">
+        <v>0</v>
+      </c>
+      <c r="P7" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>2025-12-16</t>
+        </is>
+      </c>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>2025-12-16</t>
+        </is>
+      </c>
+      <c r="S7" t="inlineStr">
+        <is>
+          <t>Corte</t>
+        </is>
+      </c>
+      <c r="T7" t="inlineStr">
+        <is>
+          <t>Ing. Fernando Silva</t>
+        </is>
+      </c>
+      <c r="U7" t="inlineStr">
+        <is>
+          <t>Operativo</t>
+        </is>
+      </c>
+      <c r="V7" t="inlineStr">
+        <is>
+          <t>media/fotos_activos/EQM-REG-002.jpg</t>
+        </is>
+      </c>
+      <c r="W7" t="inlineStr">
+        <is>
+          <t>media/qrs/QR_EQM-REG-002.png</t>
+        </is>
+      </c>
+      <c r="X7" t="inlineStr">
+        <is>
+          <t>2026-09-17 13:02</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>EQM-TRF-001</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Transformador Eléctrico Industrial 1 (60kVA)</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>FLBXON</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>FTR3-60KVA</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>SN-EQM-TRF-001</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Herramientas y Periféricos</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Transformador / Regulador</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>4A1E8D23-67BC-44F1-92EA-EQMTRF001</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>FCM180614LK2</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>I02 Maquinaria y equipo</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr"/>
+      <c r="M8" t="n">
+        <v>47577.75</v>
+      </c>
+      <c r="N8" t="n">
+        <v>2378.89</v>
+      </c>
+      <c r="O8" t="n">
+        <v>49956.64</v>
+      </c>
+      <c r="P8" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>2025-12-16</t>
+        </is>
+      </c>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>2025-12-16</t>
+        </is>
+      </c>
+      <c r="S8" t="inlineStr">
+        <is>
+          <t>Corte</t>
+        </is>
+      </c>
+      <c r="T8" t="inlineStr">
+        <is>
+          <t>Ing. Fernando Silva</t>
+        </is>
+      </c>
+      <c r="U8" t="inlineStr">
+        <is>
+          <t>Operativo</t>
+        </is>
+      </c>
+      <c r="V8" t="inlineStr">
+        <is>
+          <t>media/fotos_activos/EQM-TRF-001.jpg</t>
+        </is>
+      </c>
+      <c r="W8" t="inlineStr">
+        <is>
+          <t>media/qrs/QR_EQM-TRF-001.png</t>
+        </is>
+      </c>
+      <c r="X8" t="inlineStr">
+        <is>
+          <t>2026-09-17 13:02</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>EQM-TRF-002</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Transformador Eléctrico Industrial 2 (75kVA)</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>FLBXON</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>FTR3-75KVA</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>SN-EQM-TRF-002</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Herramientas y Periféricos</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Transformador / Regulador</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>4A1E8D23-67BC-44F1-92EA-EQMTRF002</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>FCM180614LK2</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>I02 Maquinaria y equipo</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr"/>
+      <c r="M9" t="n">
+        <v>47577.75</v>
+      </c>
+      <c r="N9" t="n">
+        <v>2378.89</v>
+      </c>
+      <c r="O9" t="n">
+        <v>49956.64</v>
+      </c>
+      <c r="P9" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>2025-12-16</t>
+        </is>
+      </c>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>2025-12-16</t>
+        </is>
+      </c>
+      <c r="S9" t="inlineStr">
+        <is>
+          <t>Corte</t>
+        </is>
+      </c>
+      <c r="T9" t="inlineStr">
+        <is>
+          <t>Ing. Fernando Silva</t>
+        </is>
+      </c>
+      <c r="U9" t="inlineStr">
+        <is>
+          <t>Operativo</t>
+        </is>
+      </c>
+      <c r="V9" t="inlineStr">
+        <is>
+          <t>media/fotos_activos/EQM-TRF-002.jpg</t>
+        </is>
+      </c>
+      <c r="W9" t="inlineStr">
+        <is>
+          <t>media/qrs/QR_EQM-TRF-002.png</t>
+        </is>
+      </c>
+      <c r="X9" t="inlineStr">
+        <is>
+          <t>2026-09-17 13:02</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>DBL-PRE-001</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Prensa Dobladora CNC 200 Toneladas (Planta Metales)</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>FLEXMAX</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>WC67K-200T/3200</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>20250110629</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Maquinaria Principal</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Prensa Dobladora</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>4A1E8D23-67BC-44F1-92EA-DBLPRE001</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>FCM180614LK2</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>I02 Maquinaria y equipo</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr"/>
+      <c r="M10" t="n">
+        <v>840868.75</v>
+      </c>
+      <c r="N10" t="n">
+        <v>42043.44</v>
+      </c>
+      <c r="O10" t="n">
+        <v>882912.1899999999</v>
+      </c>
+      <c r="P10" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>2026-02-24</t>
+        </is>
+      </c>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>2026-02-24</t>
+        </is>
+      </c>
+      <c r="S10" t="inlineStr">
+        <is>
+          <t>Doblez</t>
+        </is>
+      </c>
+      <c r="T10" t="inlineStr">
+        <is>
+          <t>Ing. Miguel Ángel Rocha</t>
+        </is>
+      </c>
+      <c r="U10" t="inlineStr">
+        <is>
+          <t>Operativo</t>
+        </is>
+      </c>
+      <c r="V10" t="inlineStr">
+        <is>
+          <t>media/fotos_activos/DBL-PRE-001.jpg</t>
+        </is>
+      </c>
+      <c r="W10" t="inlineStr">
+        <is>
+          <t>media/qrs/QR_DBL-PRE-001.png</t>
+        </is>
+      </c>
+      <c r="X10" t="inlineStr">
+        <is>
+          <t>2026-09-17 13:02</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>DBL-PRE-002</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Prensa Dobladora CNC 63 Toneladas</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>FLEXMAX</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>WC67K-63T/1600</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>2025090511</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Maquinaria Principal</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Prensa Dobladora</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>4A1E8D23-67BC-44F1-92EA-DBLPRE002</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>FCM180614LK2</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>I02 Maquinaria y equipo</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr"/>
+      <c r="M11" t="n">
+        <v>362901.25</v>
+      </c>
+      <c r="N11" t="n">
+        <v>18145.06</v>
+      </c>
+      <c r="O11" t="n">
+        <v>381046.31</v>
+      </c>
+      <c r="P11" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>2026-02-24</t>
+        </is>
+      </c>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>2026-02-24</t>
+        </is>
+      </c>
+      <c r="S11" t="inlineStr">
+        <is>
+          <t>Doblez</t>
+        </is>
+      </c>
+      <c r="T11" t="inlineStr">
+        <is>
+          <t>Ing. Miguel Ángel Rocha</t>
+        </is>
+      </c>
+      <c r="U11" t="inlineStr">
+        <is>
+          <t>Operativo</t>
+        </is>
+      </c>
+      <c r="V11" t="inlineStr">
+        <is>
+          <t>media/fotos_activos/DBL-PRE-002.jpg</t>
+        </is>
+      </c>
+      <c r="W11" t="inlineStr">
+        <is>
+          <t>media/qrs/QR_DBL-PRE-002.png</t>
+        </is>
+      </c>
+      <c r="X11" t="inlineStr">
+        <is>
+          <t>2026-09-17 13:02</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>EQM-REG-003</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Regulador Eléctrico 30kVA (380V)</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>FLBXON</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>FVR-30KVA-380V</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>S/N</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Herramientas y Periféricos</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Transformador / Regulador</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>4A1E8D23-67BC-44F1-92EA-EQMREG003</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>FCM180614LK2</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>I02 Maquinaria y equipo</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr"/>
+      <c r="M12" t="n">
+        <v>21078.75</v>
+      </c>
+      <c r="N12" t="n">
+        <v>1053.94</v>
+      </c>
+      <c r="O12" t="n">
+        <v>22132.69</v>
+      </c>
+      <c r="P12" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>2026-02-24</t>
+        </is>
+      </c>
+      <c r="R12" t="inlineStr">
+        <is>
+          <t>2026-02-24</t>
+        </is>
+      </c>
+      <c r="S12" t="inlineStr">
+        <is>
+          <t>Doblez</t>
+        </is>
+      </c>
+      <c r="T12" t="inlineStr">
+        <is>
+          <t>Ing. Fernando Silva</t>
+        </is>
+      </c>
+      <c r="U12" t="inlineStr">
+        <is>
+          <t>Operativo</t>
+        </is>
+      </c>
+      <c r="V12" t="inlineStr">
+        <is>
+          <t>media/fotos_activos/EQM-REG-003.jpg</t>
+        </is>
+      </c>
+      <c r="W12" t="inlineStr">
+        <is>
+          <t>media/qrs/QR_EQM-REG-003.png</t>
+        </is>
+      </c>
+      <c r="X12" t="inlineStr">
+        <is>
+          <t>2026-09-17 13:02</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>EQM-REG-004</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Regulador Eléctrico 20kVA (380V)</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>FLBXON</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>FVR-20KVA-380V</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>S/N</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Herramientas y Periféricos</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Transformador / Regulador</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>4A1E8D23-67BC-44F1-92EA-EQMREG004</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>FCM180614LK2</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>I02 Maquinaria y equipo</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr"/>
+      <c r="M13" t="n">
+        <v>17538.25</v>
+      </c>
+      <c r="N13" t="n">
+        <v>876.91</v>
+      </c>
+      <c r="O13" t="n">
+        <v>18415.16</v>
+      </c>
+      <c r="P13" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q13" t="inlineStr">
+        <is>
+          <t>2026-02-24</t>
+        </is>
+      </c>
+      <c r="R13" t="inlineStr">
+        <is>
+          <t>2026-02-24</t>
+        </is>
+      </c>
+      <c r="S13" t="inlineStr">
+        <is>
+          <t>Doblez</t>
+        </is>
+      </c>
+      <c r="T13" t="inlineStr">
+        <is>
+          <t>Ing. Fernando Silva</t>
+        </is>
+      </c>
+      <c r="U13" t="inlineStr">
+        <is>
+          <t>Operativo</t>
+        </is>
+      </c>
+      <c r="V13" t="inlineStr">
+        <is>
+          <t>media/fotos_activos/EQM-REG-004.jpg</t>
+        </is>
+      </c>
+      <c r="W13" t="inlineStr">
+        <is>
+          <t>media/qrs/QR_EQM-REG-004.png</t>
+        </is>
+      </c>
+      <c r="X13" t="inlineStr">
+        <is>
+          <t>2026-09-17 13:02</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>LIJ-AUT-001</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Lijadora Automática de Banda Ancha 1 Metro (SAND-R330)</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>FLEXMAX</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>SAND-R330</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>22120625121503</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Maquinaria Principal</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Lijadora / Acabados</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>4A1E8D23-67BC-44F1-92EA-LIJAUT001</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>FCM180614LK2</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>I02 Maquinaria y equipo</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr"/>
+      <c r="M14" t="n">
+        <v>0</v>
+      </c>
+      <c r="N14" t="n">
+        <v>0</v>
+      </c>
+      <c r="O14" t="n">
+        <v>0</v>
+      </c>
+      <c r="P14" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q14" t="inlineStr">
+        <is>
+          <t>2025-12-16</t>
+        </is>
+      </c>
+      <c r="R14" t="inlineStr">
+        <is>
+          <t>2025-12-16</t>
+        </is>
+      </c>
+      <c r="S14" t="inlineStr">
+        <is>
+          <t>Acabados</t>
+        </is>
+      </c>
+      <c r="T14" t="inlineStr">
+        <is>
+          <t>Téc. Jesús Ramos</t>
+        </is>
+      </c>
+      <c r="U14" t="inlineStr">
+        <is>
+          <t>Operativo</t>
+        </is>
+      </c>
+      <c r="V14" t="inlineStr">
+        <is>
+          <t>media/fotos_activos/LIJ-AUT-001.jpg</t>
+        </is>
+      </c>
+      <c r="W14" t="inlineStr">
+        <is>
+          <t>media/qrs/QR_LIJ-AUT-001.png</t>
+        </is>
+      </c>
+      <c r="X14" t="inlineStr">
+        <is>
+          <t>2026-09-17 13:02</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>LIJ-MAN-001</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Lijadora Manual de Acabados Chica (SAND-P1300)</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>FLEXMAX</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>SAND-P1300</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>22120625121506</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Herramientas y Periféricos</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Lijadora / Acabados</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>4A1E8D23-67BC-44F1-92EA-LIJMAN001</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>FCM180614LK2</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>I02 Maquinaria y equipo</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr"/>
+      <c r="M15" t="n">
+        <v>0</v>
+      </c>
+      <c r="N15" t="n">
+        <v>0</v>
+      </c>
+      <c r="O15" t="n">
+        <v>0</v>
+      </c>
+      <c r="P15" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q15" t="inlineStr">
+        <is>
+          <t>2025-12-16</t>
+        </is>
+      </c>
+      <c r="R15" t="inlineStr">
+        <is>
+          <t>2025-12-16</t>
+        </is>
+      </c>
+      <c r="S15" t="inlineStr">
+        <is>
+          <t>Acabados</t>
+        </is>
+      </c>
+      <c r="T15" t="inlineStr">
+        <is>
+          <t>Téc. Jesús Ramos</t>
+        </is>
+      </c>
+      <c r="U15" t="inlineStr">
+        <is>
+          <t>Operativo</t>
+        </is>
+      </c>
+      <c r="V15" t="inlineStr">
+        <is>
+          <t>media/fotos_activos/LIJ-MAN-001.jpg</t>
+        </is>
+      </c>
+      <c r="W15" t="inlineStr">
+        <is>
+          <t>media/qrs/QR_LIJ-MAN-001.png</t>
+        </is>
+      </c>
+      <c r="X15" t="inlineStr">
+        <is>
+          <t>2026-09-17 13:02</t>
         </is>
       </c>
     </row>

</xml_diff>